<commit_message>
Import Fenote enrolment Excel into student, teacher, and staff registries.
MayaBela reads Fenote_Raey_Enrolment_Forms.xlsx (form and register sheets),
accepts full or partial rows, ignores gold office ID columns, and writes
people through the same addStudent / addTeacher path. IDs are still issued
by the software after save.

Co-authored-by: nebila310-ship-it <nebila310-ship-it@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/fenote-raey/enrolment-forms/Fenote_Raey_Enrolment_Forms.xlsx
+++ b/docs/fenote-raey/enrolment-forms/Fenote_Raey_Enrolment_Forms.xlsx
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -622,21 +622,21 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Sheets</t>
+          <t>Import into MayaBela</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Student form / Teacher form / Admin staff form — one person at a time. Type in column B. Dropdowns are provided.</t>
+          <t xml:space="preserve">  Students directory, Teachers / Administration Staff directory, or Go-live → Import → pick this file.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Student register / Teacher register / Staff register — many people, one row each. Use this to collect a class or a hiring batch, then type into MayaBela.</t>
+          <t xml:space="preserve">  Full rows and partial rows both work. Empty rows are skipped. Gold office columns are ignored — the software still issues STU- / TCH- / QA- / HR- IDs.</t>
         </is>
       </c>
     </row>
@@ -646,52 +646,52 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Required in software (*)</t>
+          <t>Sheets</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Student: full name, gender, date of birth (DD/MM/YYYY), grade, section.</t>
+          <t xml:space="preserve">  • Student form / Teacher form / Admin staff form — one person at a time. Type in column B. Dropdowns are provided.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Teacher: full name, email, phone (the phone becomes the login).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Administrative staff: full name, email, phone, and at least one role.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="8" customHeight="1">
-      <c r="A13" s="2" t="inlineStr"/>
+          <t xml:space="preserve">  • Student register / Teacher register / Staff register — many people, one row each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="8" customHeight="1">
+      <c r="A12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Required in software (*)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>After you save in MayaBela, copy into the gold Office columns:</t>
+          <t xml:space="preserve">  Student: full name, gender, date of birth (DD/MM/YYYY), grade, section.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Student ID STU-####   Teacher ID TCH-####   Staff ID QA-/HR-/REG-/…   login   temporary password   QR / parent invite.</t>
+          <t xml:space="preserve">  Teacher: full name, email, phone (the phone becomes the login).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Do not invent IDs in Excel first. The software creates them.</t>
+          <t xml:space="preserve">  Administrative staff: full name, email, phone, and at least one role.</t>
         </is>
       </c>
     </row>
@@ -701,22 +701,46 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Photo: Insert → Pictures into the PHOTO box on the form sheet, or keep the printed 3×4 cm photo for the paper file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="8" customHeight="1">
-      <c r="A19" s="2" t="inlineStr"/>
+          <t>After you save in MayaBela, copy into the gold Office columns:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Student ID STU-####   Teacher ID TCH-####   Staff ID QA-/HR-/REG-/…   login   temporary password   QR / parent invite.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>Do not invent IDs in Excel first. The software creates them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Photo: Insert → Pictures into the PHOTO box on the form sheet, or keep the printed 3×4 cm photo for the paper file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="8" customHeight="1">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Software screens: Admin → Add Student  ·  Add Teacher  ·  Add Administration Staff</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Support: +251 911 646 444  ·  majobridgetech@gmail.com  ·  https://mayabela.pages.dev</t>
         </is>

</xml_diff>